<commit_message>
completed the materials and interactions , physics objects, simulated objects, sections. just aniimated objects, object spawners and >=3 peers
</commit_message>
<xml_diff>
--- a/Flocking Benchmark.xlsx
+++ b/Flocking Benchmark.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\711805.ADIR\source\repos\GameEngine\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF086B5F-7948-474D-A4CE-8F3ABCBE5F43}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E92844A-61D0-42D0-9912-87E3675D95D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="8340" yWindow="1850" windowWidth="28800" windowHeight="15370" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
   <si>
     <t>Brute-Force</t>
   </si>
@@ -37,6 +37,9 @@
   </si>
   <si>
     <t>Time taken per frame (ms)</t>
+  </si>
+  <si>
+    <t># boids</t>
   </si>
 </sst>
 </file>
@@ -164,7 +167,7 @@
               <a:cs typeface="+mn-cs"/>
             </a:defRPr>
           </a:pPr>
-          <a:endParaRPr lang="en-US"/>
+          <a:endParaRPr lang="en-GB"/>
         </a:p>
       </c:txPr>
     </c:title>
@@ -1452,6 +1455,9 @@
       <c r="J1" s="1"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>4</v>
+      </c>
       <c r="B2">
         <v>64</v>
       </c>

</xml_diff>